<commit_message>
Product 29 test cases commit
</commit_message>
<xml_diff>
--- a/reports/ui/ExecutionSummary.xlsx
+++ b/reports/ui/ExecutionSummary.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="27">
   <si>
     <t>Execution ID</t>
   </si>
@@ -51,7 +51,7 @@
     <t>API Response</t>
   </si>
   <si>
-    <t>CALIBO-20260831-121521</t>
+    <t>CALIBO-20261013-154441</t>
   </si>
   <si>
     <t>qa</t>
@@ -63,7 +63,7 @@
     <t>Execution Time</t>
   </si>
   <si>
-    <t>2026-08-31 12:15:21</t>
+    <t>2026-10-13 15:44:41</t>
   </si>
   <si>
     <t>Total Tests</t>
@@ -81,28 +81,19 @@
     <t>Pass Rate</t>
   </si>
   <si>
-    <t>0.00%</t>
-  </si>
-  <si>
-    <t>ProE2EWithMandatoryFieldsForDemo</t>
-  </si>
-  <si>
-    <t>FAIL</t>
-  </si>
-  <si>
-    <t>2026-08-31 12:13:02</t>
-  </si>
-  <si>
-    <t>UNKNOWN</t>
+    <t>100.00%</t>
+  </si>
+  <si>
+    <t>MaturityAssesmentTeamLevelwithSprint</t>
+  </si>
+  <si>
+    <t>PASS</t>
+  </si>
+  <si>
+    <t>2026-10-13 15:42:03</t>
   </si>
   <si>
     <t>N/A</t>
-  </si>
-  <si>
-    <t>SKIP</t>
-  </si>
-  <si>
-    <t>SKIPPED</t>
   </si>
 </sst>
 </file>
@@ -147,11 +138,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="22.3515625" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="29.03515625" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="31.4375" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="5.59765625" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="10.546875" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="18.23046875" customWidth="true" bestFit="true"/>
@@ -222,60 +213,22 @@
         <v>16</v>
       </c>
       <c r="G2" t="n" s="0">
-        <v>138.0</v>
+        <v>158.0</v>
       </c>
       <c r="H2" t="s" s="0">
         <v>26</v>
       </c>
       <c r="I2" t="n" s="0">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
       <c r="J2" t="s" s="0">
         <v>14</v>
       </c>
       <c r="K2" t="s" s="0">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="L2" t="s" s="0">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="B3" t="s" s="0">
-        <v>23</v>
-      </c>
-      <c r="C3" t="s" s="0">
-        <v>28</v>
-      </c>
-      <c r="D3" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="E3" t="s" s="0">
-        <v>25</v>
-      </c>
-      <c r="F3" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="G3" t="n" s="0">
-        <v>138.0</v>
-      </c>
-      <c r="H3" t="s" s="0">
-        <v>29</v>
-      </c>
-      <c r="I3" t="n" s="0">
-        <v>2.0</v>
-      </c>
-      <c r="J3" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="K3" t="s" s="0">
-        <v>27</v>
-      </c>
-      <c r="L3" t="s" s="0">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -329,7 +282,7 @@
         <v>17</v>
       </c>
       <c r="B6" t="n" s="0">
-        <v>3.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="7">
@@ -337,7 +290,7 @@
         <v>18</v>
       </c>
       <c r="B7" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="8">
@@ -345,7 +298,7 @@
         <v>19</v>
       </c>
       <c r="B8" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="9">
@@ -353,7 +306,7 @@
         <v>20</v>
       </c>
       <c r="B9" t="n" s="0">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
Added working test cases
</commit_message>
<xml_diff>
--- a/reports/ui/ExecutionSummary.xlsx
+++ b/reports/ui/ExecutionSummary.xlsx
@@ -51,7 +51,7 @@
     <t>API Response</t>
   </si>
   <si>
-    <t>CALIBO-20261013-154441</t>
+    <t>CALIBO-20261014-115948</t>
   </si>
   <si>
     <t>qa</t>
@@ -63,7 +63,7 @@
     <t>Execution Time</t>
   </si>
   <si>
-    <t>2026-10-13 15:44:41</t>
+    <t>2026-10-14 11:59:48</t>
   </si>
   <si>
     <t>Total Tests</t>
@@ -84,13 +84,13 @@
     <t>100.00%</t>
   </si>
   <si>
-    <t>MaturityAssesmentTeamLevelwithSprint</t>
+    <t>AddProductToRelease</t>
   </si>
   <si>
     <t>PASS</t>
   </si>
   <si>
-    <t>2026-10-13 15:42:03</t>
+    <t>2026-10-14 11:58:09</t>
   </si>
   <si>
     <t>N/A</t>
@@ -142,7 +142,7 @@
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="22.3515625" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="31.4375" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="17.60546875" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="5.59765625" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="10.546875" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="18.23046875" customWidth="true" bestFit="true"/>
@@ -213,7 +213,7 @@
         <v>16</v>
       </c>
       <c r="G2" t="n" s="0">
-        <v>158.0</v>
+        <v>98.0</v>
       </c>
       <c r="H2" t="s" s="0">
         <v>26</v>

</xml_diff>